<commit_message>
Update Risks and Activities Dashboard
</commit_message>
<xml_diff>
--- a/data/project-dashboard.xlsx
+++ b/data/project-dashboard.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF233BC7-E6BD-4A3D-B665-255D811A054A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="855" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="855" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project_Info" sheetId="1" r:id="rId1"/>
@@ -7202,10 +7202,6 @@
   </cellStyles>
   <dxfs count="35">
     <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <font>
         <color rgb="FF006100"/>
       </font>
@@ -7363,6 +7359,10 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -9404,7 +9404,7 @@
     <tableColumn id="10" xr3:uid="{9EAC2262-2A27-42A8-BB73-73F39AFC4912}" name="Schedule % Complete" dataDxfId="25" dataCellStyle="Per cent"/>
     <tableColumn id="11" xr3:uid="{B218F782-EF65-4945-9E84-E0A88975643B}" name="Performance % Complete" dataDxfId="24" dataCellStyle="Per cent"/>
     <tableColumn id="12" xr3:uid="{85C93BA9-907D-4549-9ECD-E1601A6B8FF1}" name="Total Float" dataDxfId="23"/>
-    <tableColumn id="13" xr3:uid="{C49B17F2-109E-42EB-814F-75ABCAF72ADF}" name="Critical" dataDxfId="0"/>
+    <tableColumn id="13" xr3:uid="{C49B17F2-109E-42EB-814F-75ABCAF72ADF}" name="Critical" dataDxfId="22"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -9426,17 +9426,17 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="IssuesRisksTable" displayName="IssuesRisksTable" ref="A1:I5" dataDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="IssuesRisksTable" displayName="IssuesRisksTable" ref="A1:I5" dataDxfId="21">
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="Risk ID" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Risk Description" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Impact Summary" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="Probability" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="Impact" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="Risk Level" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" name="Risk Owner" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="Mitigation" dataDxfId="14"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0500-000009000000}" name="Target Date" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="Risk ID" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Risk Description" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Impact Summary" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="Probability" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="Impact" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="Risk Level" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" name="Risk Owner" dataDxfId="14"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="Mitigation" dataDxfId="13"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0500-000009000000}" name="Target Date" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -9458,15 +9458,15 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{A2B8666E-147E-4183-82CC-79B74FF1D518}" name="SPITrendTable17" displayName="SPITrendTable17" ref="A1:J2">
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{60CDD5EE-B607-4D51-A2AC-550AB14A03F3}" name="Month"/>
-    <tableColumn id="2" xr3:uid="{76772940-DA13-40AE-BA52-917177C89224}" name="01-Feb-2026" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{F0248E2B-506D-42FB-B594-3D1B0C0B4368}" name="01-Mar-2026" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{1235EC57-E169-4937-B53F-0C4A6D4C5E0F}" name="01-Apr-2026" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{7E0642A5-711D-421D-9854-5659F4096F36}" name="01-May-2026" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{88D79C57-C3FB-4564-A7BE-EDB347046130}" name="01-Jun-2026" dataDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{FBD55C5C-8427-4396-A9A1-D8D5EEDAA0F8}" name="01-Jul-2026" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{16A53D90-2572-4B4A-B792-FF1B1888C5A4}" name="01-Aug-2026" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{153860B1-419C-48D2-8D33-F85625CFBC01}" name="01-Sep-2026" dataDxfId="5"/>
-    <tableColumn id="10" xr3:uid="{C6E67E4F-856C-4338-B620-93C903A271F9}" name="01-Oct-2026" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{76772940-DA13-40AE-BA52-917177C89224}" name="01-Feb-2026" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{F0248E2B-506D-42FB-B594-3D1B0C0B4368}" name="01-Mar-2026" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{1235EC57-E169-4937-B53F-0C4A6D4C5E0F}" name="01-Apr-2026" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{7E0642A5-711D-421D-9854-5659F4096F36}" name="01-May-2026" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{88D79C57-C3FB-4564-A7BE-EDB347046130}" name="01-Jun-2026" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{FBD55C5C-8427-4396-A9A1-D8D5EEDAA0F8}" name="01-Jul-2026" dataDxfId="6"/>
+    <tableColumn id="8" xr3:uid="{16A53D90-2572-4B4A-B792-FF1B1888C5A4}" name="01-Aug-2026" dataDxfId="5"/>
+    <tableColumn id="9" xr3:uid="{153860B1-419C-48D2-8D33-F85625CFBC01}" name="01-Sep-2026" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{C6E67E4F-856C-4338-B620-93C903A271F9}" name="01-Oct-2026" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -10120,7 +10120,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10257,10 +10257,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E6">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
       <formula>0.8</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThanOrEqual">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>